<commit_message>
Record complete QA execution time
</commit_message>
<xml_diff>
--- a/bug-reports.xlsx
+++ b/bug-reports.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Reports" sheetId="1" r:id="R2d3abe417d014b19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Reports" sheetId="1" r:id="Rd4dea31d6dd94712"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -514,7 +514,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Пугин Максим Витальевич · 11 сентября 2026 · активное время 18 минут 48 секунд</x:v>
+        <x:v>Пугин Максим Витальевич · 11 сентября 2026 · активное время 1 час 16 минут 33 секунды</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -575,13 +575,13 @@
       </x:c>
       <x:c r="C7" s="13" t="str"/>
       <x:c r="D7" s="13" t="str">
-        <x:v>14:23:24–14:30:56 МСК</x:v>
+        <x:v>14:23:24–15:28:41 МСК</x:v>
       </x:c>
       <x:c r="E7" s="13" t="str">
-        <x:v>Перерыв</x:v>
+        <x:v>Полный интервал</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
-        <x:v>исключён</x:v>
+        <x:v>5:09:01</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
@@ -796,7 +796,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc013b87fa8d4690"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra276b5a1cc61439d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>